<commit_message>
testing was done according to the text file. some pieces of code needed to be modified.
</commit_message>
<xml_diff>
--- a/HW/KiCad/AETS/AETS-CZ-NB-3L0Y7S3_vyplnena.xlsx
+++ b/HW/KiCad/AETS/AETS-CZ-NB-3L0Y7S3_vyplnena.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://schaeffler-my.sharepoint.com/personal/uiv10467_vitesco_com/Documents/Plocha/automatedelectrictestingsystem_aets/HW/KiCad/AETS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://schaeffler-my.sharepoint.com/personal/uiv10467_vitesco_com/Documents/Plocha/AETS/AETS/HW/KiCad/AETS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="416" documentId="8_{3FC1093F-7553-48B3-8AE6-5FD37BCBA7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12E260B3-D6AF-4842-B129-992678282D74}"/>
+  <xr:revisionPtr revIDLastSave="441" documentId="8_{3FC1093F-7553-48B3-8AE6-5FD37BCBA7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76507BFE-F380-494D-9AF7-96BB4CC60B69}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6ABB2B52-E43F-489D-A699-C68BCEE506EC}"/>
+    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{6ABB2B52-E43F-489D-A699-C68BCEE506EC}"/>
   </bookViews>
   <sheets>
     <sheet name="AETS-CZ-NB-3L0Y7S3" sheetId="3" r:id="rId1"/>
@@ -1832,10 +1832,10 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="81.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="56.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="90.42578125" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" customWidth="1"/>
     <col min="6" max="6" width="24.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="22.140625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.140625" customWidth="1"/>

</xml_diff>

<commit_message>
added calibration feature to init screen
</commit_message>
<xml_diff>
--- a/HW/KiCad/AETS/AETS-CZ-NB-3L0Y7S3_vyplnena.xlsx
+++ b/HW/KiCad/AETS/AETS-CZ-NB-3L0Y7S3_vyplnena.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://schaeffler-my.sharepoint.com/personal/uiv10467_vitesco_com/Documents/Plocha/AETS/AETS/HW/KiCad/AETS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="441" documentId="8_{3FC1093F-7553-48B3-8AE6-5FD37BCBA7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76507BFE-F380-494D-9AF7-96BB4CC60B69}"/>
+  <xr:revisionPtr revIDLastSave="443" documentId="8_{3FC1093F-7553-48B3-8AE6-5FD37BCBA7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE0A7C01-F265-486E-9982-52EB38A28535}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{6ABB2B52-E43F-489D-A699-C68BCEE506EC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6ABB2B52-E43F-489D-A699-C68BCEE506EC}"/>
   </bookViews>
   <sheets>
     <sheet name="AETS-CZ-NB-3L0Y7S3" sheetId="3" r:id="rId1"/>
@@ -4165,4 +4165,10 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{3f3ac890-09a1-47d3-8d04-15427d7fec91}" enabled="1" method="Standard" siteId="{39b77101-99b7-41c9-8d6a-7794b9d48476}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>